<commit_message>
Replace scanone with multi-QTL for main text
</commit_message>
<xml_diff>
--- a/Data/tsu_kas_pheno_geno/TsuKas_RIL_ovule_counts.xlsx
+++ b/Data/tsu_kas_pheno_geno/TsuKas_RIL_ovule_counts.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madisonplunkert/Documents/Conner Lab/Tsu Kas QTL Mapping/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madisonplunkert/Documents/GitHub/Stamen-loss-2025/Data/tsu_kas_pheno_geno/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C03807A-D7D7-AE4E-9038-7878061026E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29FFCE2-3015-C54E-A50C-AE36F85435A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="20580" windowHeight="18840" xr2:uid="{46830B3E-A9D1-8C43-BB40-1E6B200BE5C9}"/>
+    <workbookView xWindow="5580" yWindow="740" windowWidth="20580" windowHeight="16860" xr2:uid="{46830B3E-A9D1-8C43-BB40-1E6B200BE5C9}"/>
   </bookViews>
   <sheets>
     <sheet name="RIL Set 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentCalc="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
   <si>
     <t>tube.num</t>
   </si>
@@ -111,9 +111,6 @@
   </si>
   <si>
     <t>1640/9</t>
-  </si>
-  <si>
-    <t>CS1640/8</t>
   </si>
   <si>
     <t>MeanOvuleNo</t>
@@ -487,7 +484,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -36438,7 +36435,7 @@
         <v>1284</v>
       </c>
       <c r="B1962" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C1962">
         <f t="shared" si="30"/>
@@ -38037,7 +38034,7 @@
         <v>96914</v>
       </c>
       <c r="C2050">
-        <f t="shared" ref="C2050:C2113" si="32">AVERAGE(D2050:G2050)</f>
+        <f t="shared" ref="C2050:C2052" si="32">AVERAGE(D2050:G2050)</f>
         <v>72</v>
       </c>
       <c r="D2050">

</xml_diff>